<commit_message>
Thu Sep 24 14:39:15 EEST 2026
</commit_message>
<xml_diff>
--- a/VFS_Portugal/VFS_Accounts_Exports.xlsx
+++ b/VFS_Portugal/VFS_Accounts_Exports.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -454,10 +454,10 @@
         <v>Alexandria</v>
       </c>
       <c r="E2" t="str">
-        <v>Appeal</v>
+        <v>Short Term Visa</v>
       </c>
       <c r="F2" t="str">
-        <v>Appeal against the decision</v>
+        <v>Tourism</v>
       </c>
       <c r="G2" t="str">
         <v>Visible</v>
@@ -495,19 +495,19 @@
         <v>Alexandria</v>
       </c>
       <c r="E3" t="str">
-        <v>Appeal</v>
+        <v>Short Term Visa</v>
       </c>
       <c r="F3" t="str">
-        <v>Appeal against the decision</v>
+        <v>Tourism</v>
       </c>
       <c r="G3" t="str">
-        <v>Visible</v>
+        <v>Headless</v>
       </c>
       <c r="H3" t="str">
-        <v>2</v>
+        <v/>
       </c>
       <c r="I3" t="str">
-        <v>00/00/05/20</v>
+        <v/>
       </c>
       <c r="J3" t="str">
         <v/>
@@ -519,12 +519,94 @@
         <v>1</v>
       </c>
       <c r="M3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>yallavisa4@gmail.com</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Yallavisa@@123</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Alexandria</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Appeal</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Appeal against the decision</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v>00/00/00/20</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Refresh</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>sirmohamedh@gmail.com</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Moed!vsfG@26</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Egypt</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Alexandria</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Appeal</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Appeal against the decision</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Headless</v>
+      </c>
+      <c r="H5" t="str">
+        <v>2</v>
+      </c>
+      <c r="I5" t="str">
+        <v>00/00/00/20</v>
+      </c>
+      <c r="J5" t="str">
+        <v>2</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>